<commit_message>
Language Screenshots Drop Zone
</commit_message>
<xml_diff>
--- a/Data/BugTracker/BugTracker.xlsx
+++ b/Data/BugTracker/BugTracker.xlsx
@@ -97,7 +97,7 @@
     <x:t>Compliance</x:t>
   </x:si>
   <x:si>
-    <x:t>[FR, ES] SSS</x:t>
+    <x:t>[FR, DE, ES] SSS</x:t>
   </x:si>
   <x:si>
     <x:t>SSSS</x:t>
@@ -124,7 +124,7 @@
     <x:t>2</x:t>
   </x:si>
   <x:si>
-    <x:t>hhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhh</x:t>
+    <x:t>[FR, DE, ES] hhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhh</x:t>
   </x:si>
   <x:si>
     <x:t>dfgdfgd</x:t>
@@ -139,64 +139,67 @@
     <x:t>3</x:t>
   </x:si>
   <x:si>
+    <x:t>[FR, IT, DE, ES] WWWWWWWWWWWWWWWWWWWWWWWWW</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WWWWWWWWWWWWWWWWWWWWWWW</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WWWWWWWWWWWWWWWWWWWWWWWW</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ready To Vet</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ghjgjghjgj</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WWWWWWWWW</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WWWWWWW</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Approved</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Inconsistent Translation</x:t>
+  </x:si>
+  <x:si>
+    <x:t>[IT, DE, ES]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Shortening</x:t>
+  </x:si>
+  <x:si>
+    <x:t>zdhhdhdh</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fjfgjgjsgj</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sjfgjgjgj</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WWWWWWWWWWWWWWW</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WWWWWWWWWWWWWWWWWWWW</x:t>
+  </x:si>
+  <x:si>
     <x:t>WWWWWWWWWWWWWWWWWWWWWWWWW</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WWWWWWWWWWWWWWWWWWWWWWW</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WWWWWWWWWWWWWWWWWWWWWWWW</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ready To Vet</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ghjgjghjgj</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WWWWWWWWW</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WWWWWWW</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Approved</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Inconsistent Translation</x:t>
-  </x:si>
-  <x:si>
-    <x:t>[IT, DE, ES]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Shortening</x:t>
-  </x:si>
-  <x:si>
-    <x:t>zdhhdhdh</x:t>
-  </x:si>
-  <x:si>
-    <x:t>fjfgjgjsgj</x:t>
-  </x:si>
-  <x:si>
-    <x:t>sjfgjgjgj</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WWWWWWWWWWWWWWW</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WWWWWWWWWWWWWWWWWWWW</x:t>
   </x:si>
   <x:si>
     <x:t>Duplicate</x:t>
@@ -557,10 +560,12 @@
     <x:col min="2" max="2" width="9.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.996339" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="22.710625" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="110.996339" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="121.567768" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="45.996339" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="49.996339" style="0" customWidth="1"/>
-    <x:col min="8" max="11" width="11.853482" style="0" customWidth="1"/>
+    <x:col min="8" max="9" width="11.853482" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="8.282054" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="11.853482" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="12.710625" style="0" customWidth="1"/>
     <x:col min="13" max="13" width="22.424911" style="0" customWidth="1"/>
     <x:col min="14" max="15" width="21.567768" style="0" customWidth="1"/>
@@ -674,7 +679,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="J2" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="K2" s="0" t="s">
         <x:v>29</x:v>
@@ -810,16 +815,16 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J4" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="K4" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="L4" s="0" t="s">
         <x:v>44</x:v>
@@ -1091,7 +1096,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="G8" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H8" s="0" t="s">
         <x:v>29</x:v>
@@ -1106,7 +1111,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="L8" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="M8" s="0" t="s">
         <x:v>33</x:v>

</xml_diff>